<commit_message>
Toplu Arıza Kontrol sayfası - Streamlit'e entegre edildi
- Yeni sayfa: Toplu Arıza Kontrol (Kurum İşleri menüsü altında)
- Düzenlenebilir router tablosu (IP, Kullanıcı Adı, Şifre, Açıklama)
- Excel dosyasından otomatik yükleme özelliği
- Telnet ile router kontrolleri (VLAN, ARP, WLC/EBA, Donanım)
- Detaylı kontrol sonuçları ve raporlama
- Menu config güncellemesi
</commit_message>
<xml_diff>
--- a/toplu_ariza_kontrol/ariza_listesi.xlsx
+++ b/toplu_ariza_kontrol/ariza_listesi.xlsx
@@ -653,17 +653,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>VLAN10-Yonetim interneti yok (YOK); VLAN11-Tahta interneti yok (YOK); VLAN20-Idare interneti yok (YOK); VLAN30-Ogretmen interneti yok (YOK); VLAN40-BT interneti yok (YOK); VLAN50-Tablet interneti yok (YOK); VLAN60-Aktivasyon interneti yok (YOK); Hicbir VLAN'in interneti yok AMA router'in gercek IP'si (95.1.14.16) internete cikabiliyor - sorun MPLS/router degil, switch/VLAN/DHCP seviyesinde olabilir; WLC erisimi yok (YOK); EBA erisimi yok (YOK); VLAN10-Yonetim interface DOWN (Router-Switch Up-Link kablo sorunu olabilir); VLAN11-Tahta interface DOWN (Router-Switch Up-Link kablo sorunu olabilir); VLAN20-Idare interface DOWN (Router-Switch Up-Link kablo sorunu olabilir); VLAN30-Ogretmen interface DOWN (Router-Switch Up-Link kablo sorunu olabilir); VLAN40-BT interface DOWN (Router-Switch Up-Link kablo sorunu olabilir); VLAN50-Tablet interface DOWN (Router-Switch Up-Link kablo sorunu olabilir); VLAN60-Aktivasyon interface DOWN (Router-Switch Up-Link kablo sorunu olabilir)</t>
+          <t>Sorun yok</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>172.22.114.8</t>
+          <t>172.22.242.106</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>56.04.142-GOZPINAR-IMKB-Y-RO</t>
+          <t>49.04.142-MEHMET-AKIF-ERS-RO</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -683,75 +683,75 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
+          <t>VAR</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>VAR</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>VAR</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>VAR</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>VAR</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>VAR</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>VAR</t>
+        </is>
+      </c>
+      <c r="Q2" t="n">
+        <v>11</v>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>VAR</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>VAR</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>VAR</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
           <t>YOK</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>YOK</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>YOK</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>YOK</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>YOK</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>YOK</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>YOK</t>
-        </is>
-      </c>
-      <c r="Q2" t="n">
-        <v>9</v>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>YOK</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>YOK</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>VAR</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
         <is>
           <t>-</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>YOK</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>VLAN10-Yonetim, VLAN11-Tahta, VLAN20-Idare, VLAN30-Ogretmen, VLAN40-BT, VLAN50-Tablet, VLAN60-Aktivasyon</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -762,337 +762,13 @@
       <c r="Z2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Sorun yok</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>172.22.5.0</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>27.03.192-YESILYURT-SEHIT-RO</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>ERISIM VAR</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>HUAWEI</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="Q3" t="n">
-        <v>15</v>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>YOK</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>YOK</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr"/>
+      <c r="B3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Router donanim/kart alarmi tespit edildi (SRU dahil, seviye:Major - 'display device'/'display alarm active' ciktisina bakin, router ariza yapmis olabilir)</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>172.22.160.157</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>55.09.116-ATATURK-ORTAOKU-RO</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>ERISIM VAR</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>HUAWEI</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="Q4" t="n">
-        <v>37</v>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>YOK</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>VAR - Major (ARIZALI OLABILIR)</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr"/>
+      <c r="B4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Sorun yok</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>172.22.64.94</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>06.18.265-NURI-PAKDIL-ANA-RO</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>ERISIM VAR</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>CISCO</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q5" t="n">
-        <v>83</v>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>YOK</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>VAR</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>N/A (Cisco'da kontrol edilmiyor)</t>
-        </is>
-      </c>
-      <c r="Z5" t="inlineStr"/>
+      <c r="B5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="2" t="n"/>

</xml_diff>